<commit_message>
Corrida | SFE-GTOT | 2026-03-16 10:05:30.245394
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GTOT_out.xlsx
+++ b/indicadores/SFE-GTOT_out.xlsx
@@ -8,13 +8,14 @@
   <sheets>
     <sheet name="Portada" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Correlograma" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Referencias" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Correlograma" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="559">
   <si>
     <t xml:space="preserve"/>
   </si>
@@ -103,13 +104,13 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">02/02/2026</t>
+    <t xml:space="preserve">16/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">pcohan</t>
+    <t xml:space="preserve">ysonder</t>
   </si>
   <si>
     <t xml:space="preserve">fecha</t>
@@ -1571,6 +1572,63 @@
   </si>
   <si>
     <t xml:space="preserve">2030.12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referencias de las series incluidas en la hoja Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original | serie de datos brutos transformados, se importa directo desde base de datos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_normal | serie original con 12 forecasts obtenidos del mejor modelo ARIMA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_optimista | serie original con 12 forecasts, intervalo y límite optimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a_original_fct_pesimista | serie original con 12 forecasts, intervalo y límite pesimista</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b_d16 | salida D16 del X13-ARIMA-SEATS con los factores estacionales de la serie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c_c17 | salida C17 del X13-ARIMA-SEATS con pesos del irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_d12 | salida D12 del X13-ARIMA-SEATS con el componente tendencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_129600 | tendencia HP de largo plazo con un lambda de 129.600</t>
+  </si>
+  <si>
+    <t xml:space="preserve">d_hp_200 | suavizado con filtro HP usando lambda de 200, sirve para determinar PG automáticos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">e_ajustada | serie ajustada por estacionalidad usando el mejor modelo (LOG o NIV según el caso)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">f_filtrada | serie ajustada por estacionalidad y corregida por irregularidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final | serie f_filtrada con o sin suavizado 2x2 según el caso (es la vieja española)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">g_final_fct_normal | a_original_fct ajustada por D16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_tcml | tasas de cambio mensual logarítmicas de la serie g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_var_interanual | variaciones interanuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gg_final_var_mensual | variaciones mensuales de g_final</t>
+  </si>
+  <si>
+    <t xml:space="preserve">h_irregular | g_final/d_d12 componente irregular</t>
+  </si>
+  <si>
+    <t xml:space="preserve">i_dt | g_final/d_hp_129600 desvíos respecto de la tendencia</t>
   </si>
   <si>
     <t xml:space="preserve">Coeficientes de correlación de TCML del ICA-SFE y serie específica</t>
@@ -2167,7 +2225,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.519620154007639</v>
+        <v>0.521821113801313</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2225,7 +2283,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.270005104450922</v>
+        <v>0.272297274808843</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2295,7 +2353,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00587574007908572</v>
+        <v>0.00723174681910259</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2325,7 +2383,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000000127230938150147</v>
+        <v>0.000000174646187137664</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -28125,6 +28183,112 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>534</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>537</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -28133,7 +28297,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>519</v>
+        <v>538</v>
       </c>
       <c r="B2" s="1"/>
     </row>
@@ -28143,160 +28307,160 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>520</v>
+        <v>539</v>
       </c>
       <c r="B4" s="1"/>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>521</v>
+        <v>540</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0480895251572145</v>
+        <v>-0.0473320425647825</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>522</v>
+        <v>541</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.012460625319182</v>
+        <v>-0.0124800662989043</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>523</v>
+        <v>542</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.00390931839840585</v>
+        <v>-0.00435600359128801</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>524</v>
+        <v>543</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0340359464494571</v>
+        <v>0.0328689423559183</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>525</v>
+        <v>544</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.103182995344933</v>
+        <v>0.102089712465314</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>526</v>
+        <v>545</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.177900812850999</v>
+        <v>0.178706102268139</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>527</v>
+        <v>546</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.271561567507873</v>
+        <v>0.274154188382959</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>528</v>
+        <v>547</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.376917960840308</v>
+        <v>0.379271239176116</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>529</v>
+        <v>548</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.473735521993761</v>
+        <v>0.475455524851718</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>530</v>
+        <v>549</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.519620154007639</v>
+        <v>0.521821113801313</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>531</v>
+        <v>550</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.48769852064974</v>
+        <v>0.489818610490744</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>532</v>
+        <v>551</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.437729949563694</v>
+        <v>0.43669752381432</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>533</v>
+        <v>552</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.422217339970633</v>
+        <v>0.419066016522816</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>534</v>
+        <v>553</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.397670355584912</v>
+        <v>0.395704919652296</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>535</v>
+        <v>554</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.359385872620544</v>
+        <v>0.359747393622085</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>536</v>
+        <v>555</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.336994832114522</v>
+        <v>0.338736488986441</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>537</v>
+        <v>556</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.337509751144771</v>
+        <v>0.337982610342035</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>538</v>
+        <v>557</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.351294255822548</v>
+        <v>0.351475302206436</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>539</v>
+        <v>558</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.325603105763408</v>
+        <v>0.325403118317211</v>
       </c>
     </row>
     <row r="24">
@@ -28548,13 +28712,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C468F57A-8A71-401D-AE3A-72B464E5F823}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56B20B6D-4304-4806-B770-B5AB493B4619}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4301C881-4A8A-472D-8D41-CE6C47894638}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E555F74-1A61-45BA-8876-AB93EC757FA0}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DDEA750-CB7A-41AC-95AC-FDA4710B72AB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E51999F0-B227-40B2-8EBC-080420B41B97}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-GTOT | 2026-03-17 09:55:54.239936
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GTOT_out.xlsx
+++ b/indicadores/SFE-GTOT_out.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">16/03/2026</t>
+    <t xml:space="preserve">17/03/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -28712,13 +28712,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{56B20B6D-4304-4806-B770-B5AB493B4619}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B428B307-3A6C-4A9F-A235-B440FEE3B37F}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1E555F74-1A61-45BA-8876-AB93EC757FA0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40ED13E0-86B2-41A1-9FF9-3AF53D162084}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E51999F0-B227-40B2-8EBC-080420B41B97}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64DADA05-4727-4B8C-B5D2-ABED4C273ADE}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-GTOT | 2026-04-06 09:14:01.075195
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GTOT_out.xlsx
+++ b/indicadores/SFE-GTOT_out.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">17/03/2026</t>
+    <t xml:space="preserve">06/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2225,7 +2225,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.521821113801313</v>
+        <v>0.520239454917434</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2283,7 +2283,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.272297274808843</v>
+        <v>0.270649090452789</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2353,7 +2353,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00723174681910259</v>
+        <v>0.00682389065620887</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2383,7 +2383,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000000174646187137664</v>
+        <v>0.000000175928169327995</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -28316,7 +28316,7 @@
         <v>540</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0473320425647825</v>
+        <v>-0.0464052065461866</v>
       </c>
     </row>
     <row r="6">
@@ -28324,7 +28324,7 @@
         <v>541</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0124800662989043</v>
+        <v>-0.0120790136910358</v>
       </c>
     </row>
     <row r="7">
@@ -28332,7 +28332,7 @@
         <v>542</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.00435600359128801</v>
+        <v>-0.00399018076471317</v>
       </c>
     </row>
     <row r="8">
@@ -28340,7 +28340,7 @@
         <v>543</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0328689423559183</v>
+        <v>0.0334338672018747</v>
       </c>
     </row>
     <row r="9">
@@ -28348,7 +28348,7 @@
         <v>544</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.102089712465314</v>
+        <v>0.102072911979075</v>
       </c>
     </row>
     <row r="10">
@@ -28356,7 +28356,7 @@
         <v>545</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.178706102268139</v>
+        <v>0.178879409912402</v>
       </c>
     </row>
     <row r="11">
@@ -28364,7 +28364,7 @@
         <v>546</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.274154188382959</v>
+        <v>0.275182498727096</v>
       </c>
     </row>
     <row r="12">
@@ -28372,7 +28372,7 @@
         <v>547</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.379271239176116</v>
+        <v>0.379867193495642</v>
       </c>
     </row>
     <row r="13">
@@ -28380,7 +28380,7 @@
         <v>548</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.475455524851718</v>
+        <v>0.474671035481603</v>
       </c>
     </row>
     <row r="14">
@@ -28388,7 +28388,7 @@
         <v>549</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.521821113801313</v>
+        <v>0.520239454917434</v>
       </c>
     </row>
     <row r="15">
@@ -28396,7 +28396,7 @@
         <v>550</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.489818610490744</v>
+        <v>0.488780139940694</v>
       </c>
     </row>
     <row r="16">
@@ -28404,7 +28404,7 @@
         <v>551</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.43669752381432</v>
+        <v>0.436563144008409</v>
       </c>
     </row>
     <row r="17">
@@ -28412,7 +28412,7 @@
         <v>552</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.419066016522816</v>
+        <v>0.419092958207714</v>
       </c>
     </row>
     <row r="18">
@@ -28420,7 +28420,7 @@
         <v>553</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.395704919652296</v>
+        <v>0.396377680129619</v>
       </c>
     </row>
     <row r="19">
@@ -28428,7 +28428,7 @@
         <v>554</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.359747393622085</v>
+        <v>0.361399460874888</v>
       </c>
     </row>
     <row r="20">
@@ -28436,7 +28436,7 @@
         <v>555</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.338736488986441</v>
+        <v>0.340707429452277</v>
       </c>
     </row>
     <row r="21">
@@ -28444,7 +28444,7 @@
         <v>556</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.337982610342035</v>
+        <v>0.338995960874575</v>
       </c>
     </row>
     <row r="22">
@@ -28452,7 +28452,7 @@
         <v>557</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.351475302206436</v>
+        <v>0.351546574953138</v>
       </c>
     </row>
     <row r="23">
@@ -28460,7 +28460,7 @@
         <v>558</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.325403118317211</v>
+        <v>0.325878738925914</v>
       </c>
     </row>
     <row r="24">
@@ -28712,13 +28712,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B428B307-3A6C-4A9F-A235-B440FEE3B37F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E9A597BF-E8B6-4F34-966A-D73E5FD19C37}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{40ED13E0-86B2-41A1-9FF9-3AF53D162084}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90674A89-D862-4548-BACE-8248202A1657}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{64DADA05-4727-4B8C-B5D2-ABED4C273ADE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABDF8F4D-7ECE-4A23-AB9F-2C0782529F20}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-GTOT | 2026-04-07 08:22:47.728568
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GTOT_out.xlsx
+++ b/indicadores/SFE-GTOT_out.xlsx
@@ -50,7 +50,7 @@
     <t xml:space="preserve">Sector</t>
   </si>
   <si>
-    <t xml:space="preserve">Recursos y gastos del sector público de la provincia de Santa Fe</t>
+    <t xml:space="preserve">Recursos y gastos del sector público</t>
   </si>
   <si>
     <t xml:space="preserve">Modelo</t>
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">06/04/2026</t>
+    <t xml:space="preserve">07/04/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2353,7 +2353,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00682389065620887</v>
+        <v>0.00683088200265222</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2383,7 +2383,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.000000175928169327995</v>
+        <v>0.00000017744083413387</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -28488,237 +28488,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E9A597BF-E8B6-4F34-966A-D73E5FD19C37}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{90674A89-D862-4548-BACE-8248202A1657}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ABDF8F4D-7ECE-4A23-AB9F-2C0782529F20}"/>
 </file>
</xml_diff>

<commit_message>
Corrida | SFE-GTOT | 2026-06-01 10:34:18.421014
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GTOT_out.xlsx
+++ b/indicadores/SFE-GTOT_out.xlsx
@@ -104,7 +104,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">07/04/2026</t>
+    <t xml:space="preserve">01/06/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2225,7 +2225,7 @@
       <c r="B9"/>
       <c r="C9"/>
       <c r="D9" t="n">
-        <v>0.520239454917434</v>
+        <v>0.52077399714151</v>
       </c>
       <c r="E9"/>
       <c r="F9"/>
@@ -2283,7 +2283,7 @@
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13" t="n">
-        <v>0.270649090452789</v>
+        <v>0.271205556098745</v>
       </c>
       <c r="E13"/>
       <c r="F13"/>
@@ -2353,7 +2353,7 @@
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18" t="n">
-        <v>0.00683088200265222</v>
+        <v>0.00520791273964513</v>
       </c>
       <c r="E18"/>
       <c r="F18"/>
@@ -2383,7 +2383,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.00000017744083413387</v>
+        <v>0.000000090515001268009</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -28316,7 +28316,7 @@
         <v>540</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0464052065461866</v>
+        <v>-0.0469529625329635</v>
       </c>
     </row>
     <row r="6">
@@ -28324,7 +28324,7 @@
         <v>541</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0120790136910358</v>
+        <v>-0.00807051357772859</v>
       </c>
     </row>
     <row r="7">
@@ -28332,7 +28332,7 @@
         <v>542</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.00399018076471317</v>
+        <v>-0.00317666303986892</v>
       </c>
     </row>
     <row r="8">
@@ -28340,7 +28340,7 @@
         <v>543</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0334338672018747</v>
+        <v>0.0355605849686201</v>
       </c>
     </row>
     <row r="9">
@@ -28348,7 +28348,7 @@
         <v>544</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.102072911979075</v>
+        <v>0.10560988089219</v>
       </c>
     </row>
     <row r="10">
@@ -28356,7 +28356,7 @@
         <v>545</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.178879409912402</v>
+        <v>0.177025249250428</v>
       </c>
     </row>
     <row r="11">
@@ -28364,7 +28364,7 @@
         <v>546</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.275182498727096</v>
+        <v>0.271221679647494</v>
       </c>
     </row>
     <row r="12">
@@ -28372,7 +28372,7 @@
         <v>547</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.379867193495642</v>
+        <v>0.380068332551282</v>
       </c>
     </row>
     <row r="13">
@@ -28380,7 +28380,7 @@
         <v>548</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.474671035481603</v>
+        <v>0.47577084352192</v>
       </c>
     </row>
     <row r="14">
@@ -28388,7 +28388,7 @@
         <v>549</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.520239454917434</v>
+        <v>0.52077399714151</v>
       </c>
     </row>
     <row r="15">
@@ -28396,7 +28396,7 @@
         <v>550</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.488780139940694</v>
+        <v>0.493218107540941</v>
       </c>
     </row>
     <row r="16">
@@ -28404,7 +28404,7 @@
         <v>551</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.436563144008409</v>
+        <v>0.439859845451064</v>
       </c>
     </row>
     <row r="17">
@@ -28412,7 +28412,7 @@
         <v>552</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.419092958207714</v>
+        <v>0.417971169012904</v>
       </c>
     </row>
     <row r="18">
@@ -28420,7 +28420,7 @@
         <v>553</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.396377680129619</v>
+        <v>0.398872962384823</v>
       </c>
     </row>
     <row r="19">
@@ -28428,7 +28428,7 @@
         <v>554</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.361399460874888</v>
+        <v>0.363075583755783</v>
       </c>
     </row>
     <row r="20">
@@ -28436,7 +28436,7 @@
         <v>555</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.340707429452277</v>
+        <v>0.331510539619195</v>
       </c>
     </row>
     <row r="21">
@@ -28444,7 +28444,7 @@
         <v>556</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.338995960874575</v>
+        <v>0.329116431575633</v>
       </c>
     </row>
     <row r="22">
@@ -28452,7 +28452,7 @@
         <v>557</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.351546574953138</v>
+        <v>0.350521814195453</v>
       </c>
     </row>
     <row r="23">
@@ -28460,7 +28460,7 @@
         <v>558</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.325878738925914</v>
+        <v>0.327309154105194</v>
       </c>
     </row>
     <row r="24">

</xml_diff>

<commit_message>
Corrida | SFE-GTOT | 2026-07-02 10:00:38.20061
</commit_message>
<xml_diff>
--- a/indicadores/SFE-GTOT_out.xlsx
+++ b/indicadores/SFE-GTOT_out.xlsx
@@ -110,7 +110,7 @@
     <t xml:space="preserve">Fecha</t>
   </si>
   <si>
-    <t xml:space="preserve">24/06/2026</t>
+    <t xml:space="preserve">02/07/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Usuario</t>
@@ -2259,7 +2259,7 @@
       <c r="B11"/>
       <c r="C11"/>
       <c r="D11" t="n">
-        <v>0.521747064223895</v>
+        <v>0.521910947523055</v>
       </c>
       <c r="E11"/>
       <c r="F11"/>
@@ -2317,7 +2317,7 @@
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15" t="n">
-        <v>0.272219999026253</v>
+        <v>0.272391037144412</v>
       </c>
       <c r="E15"/>
       <c r="F15"/>
@@ -2387,7 +2387,7 @@
       <c r="B20"/>
       <c r="C20"/>
       <c r="D20" t="n">
-        <v>0.0016377226384938</v>
+        <v>0.00160402701001223</v>
       </c>
       <c r="E20"/>
       <c r="F20"/>
@@ -2417,7 +2417,7 @@
       <c r="B22"/>
       <c r="C22"/>
       <c r="D22" t="n">
-        <v>0.00000393379718379444</v>
+        <v>0.0000040586287599384</v>
       </c>
       <c r="E22"/>
       <c r="F22"/>
@@ -28506,7 +28506,7 @@
         <v>542</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>-0.0489331703350327</v>
+        <v>-0.0489819400621481</v>
       </c>
     </row>
     <row r="6">
@@ -28514,7 +28514,7 @@
         <v>543</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>-0.0178334403182965</v>
+        <v>-0.0177092021587065</v>
       </c>
     </row>
     <row r="7">
@@ -28522,7 +28522,7 @@
         <v>544</v>
       </c>
       <c r="B7" s="1" t="n">
-        <v>-0.00317282872930198</v>
+        <v>-0.00312861857453323</v>
       </c>
     </row>
     <row r="8">
@@ -28530,7 +28530,7 @@
         <v>545</v>
       </c>
       <c r="B8" s="1" t="n">
-        <v>0.0259536141338238</v>
+        <v>0.0258384944180484</v>
       </c>
     </row>
     <row r="9">
@@ -28538,7 +28538,7 @@
         <v>546</v>
       </c>
       <c r="B9" s="1" t="n">
-        <v>0.0812379128344061</v>
+        <v>0.0811342131160096</v>
       </c>
     </row>
     <row r="10">
@@ -28546,7 +28546,7 @@
         <v>547</v>
       </c>
       <c r="B10" s="1" t="n">
-        <v>0.164345501129237</v>
+        <v>0.164306464438191</v>
       </c>
     </row>
     <row r="11">
@@ -28554,7 +28554,7 @@
         <v>548</v>
       </c>
       <c r="B11" s="1" t="n">
-        <v>0.26694735306013</v>
+        <v>0.267005178244489</v>
       </c>
     </row>
     <row r="12">
@@ -28562,7 +28562,7 @@
         <v>549</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>0.368662798722981</v>
+        <v>0.368894736927612</v>
       </c>
     </row>
     <row r="13">
@@ -28570,7 +28570,7 @@
         <v>550</v>
       </c>
       <c r="B13" s="1" t="n">
-        <v>0.468445526159729</v>
+        <v>0.46874792429155</v>
       </c>
     </row>
     <row r="14">
@@ -28578,7 +28578,7 @@
         <v>551</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>0.521747064223895</v>
+        <v>0.521910947523055</v>
       </c>
     </row>
     <row r="15">
@@ -28586,7 +28586,7 @@
         <v>552</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>0.482342462699583</v>
+        <v>0.482353652460072</v>
       </c>
     </row>
     <row r="16">
@@ -28594,7 +28594,7 @@
         <v>553</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>0.426869343536061</v>
+        <v>0.426729000336219</v>
       </c>
     </row>
     <row r="17">
@@ -28602,7 +28602,7 @@
         <v>554</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>0.406392199682106</v>
+        <v>0.406063860305864</v>
       </c>
     </row>
     <row r="18">
@@ -28610,7 +28610,7 @@
         <v>555</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>0.372175737317605</v>
+        <v>0.371887081104697</v>
       </c>
     </row>
     <row r="19">
@@ -28618,7 +28618,7 @@
         <v>556</v>
       </c>
       <c r="B19" s="1" t="n">
-        <v>0.333624894425839</v>
+        <v>0.333523215772598</v>
       </c>
     </row>
     <row r="20">
@@ -28626,7 +28626,7 @@
         <v>557</v>
       </c>
       <c r="B20" s="1" t="n">
-        <v>0.321064208185525</v>
+        <v>0.320997045201466</v>
       </c>
     </row>
     <row r="21">
@@ -28634,7 +28634,7 @@
         <v>558</v>
       </c>
       <c r="B21" s="1" t="n">
-        <v>0.324960221877963</v>
+        <v>0.324876120446659</v>
       </c>
     </row>
     <row r="22">
@@ -28642,7 +28642,7 @@
         <v>559</v>
       </c>
       <c r="B22" s="1" t="n">
-        <v>0.331478639808259</v>
+        <v>0.331483090489914</v>
       </c>
     </row>
     <row r="23">
@@ -28650,7 +28650,7 @@
         <v>560</v>
       </c>
       <c r="B23" s="1" t="n">
-        <v>0.303778694654535</v>
+        <v>0.303845124238836</v>
       </c>
     </row>
     <row r="24">
@@ -28678,237 +28678,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100C5B9F2161CEE1040BBC03CB11300495F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="a7cec21613a3259523bdab11a1e26aca">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b5dd4176-d247-4204-85b8-921214f3ccea" xmlns:ns3="359b39ce-e1f9-4933-8424-33b611e6fdcd" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="68943c349d3a016936c8f8cb3335004b" ns2:_="" ns3:_="">
-    <xsd:import namespace="b5dd4176-d247-4204-85b8-921214f3ccea"/>
-    <xsd:import namespace="359b39ce-e1f9-4933-8424-33b611e6fdcd"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b5dd4176-d247-4204-85b8-921214f3ccea" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Etiquetas de imagen" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="01529062-7a8b-4d76-943d-e0db5644ee6d" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="359b39ce-e1f9-4933-8424-33b611e6fdcd" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{c9b73259-0823-4f05-8927-4a40ee49fbe1}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="359b39ce-e1f9-4933-8424-33b611e6fdcd">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de contenido"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="359b39ce-e1f9-4933-8424-33b611e6fdcd" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b5dd4176-d247-4204-85b8-921214f3ccea">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E09B7BFB-1AAF-4138-BEB0-32536CA7598E}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A2DD98BD-4D35-4084-B584-96354841D919}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A5A5443-81C6-41C9-90D2-BB9766E2405D}"/>
 </file>
</xml_diff>